<commit_message>
UI: added direct call button to header (+233 571 386600)
</commit_message>
<xml_diff>
--- a/backend/product_upload_template.xlsx
+++ b/backend/product_upload_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/realkofi.d/Documents/Development/expert-website/expert-v2/backend/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/realkofi.d/Documents/Development/expert-v2/backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31C45A2-221A-B645-8090-8A6A7790F0E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD18017-A380-054E-BEF4-7A00070DB570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40" yWindow="7080" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inventory Template" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Name</t>
   </si>
@@ -34,18 +34,9 @@
     <t>Stock</t>
   </si>
   <si>
-    <t>Category_ID</t>
-  </si>
-  <si>
-    <t>Subcategory_ID</t>
-  </si>
-  <si>
     <t>Brand</t>
   </si>
   <si>
-    <t>Color</t>
-  </si>
-  <si>
     <t>Dimensions</t>
   </si>
   <si>
@@ -58,58 +49,62 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Modern Office Desk</t>
-  </si>
-  <si>
-    <t>FUR-DK-005</t>
-  </si>
-  <si>
-    <t>Oak</t>
-  </si>
-  <si>
-    <t>140x70x75cm</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
-    <t>https://photos.app.goo.gl/example3</t>
-  </si>
-  <si>
-    <t>Minimalist oak wood desk with cable management.</t>
-  </si>
-  <si>
-    <t>Sub Furniture</t>
-  </si>
-  <si>
-    <t>COZYHOME</t>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Subcategory</t>
+  </si>
+  <si>
+    <t>Material</t>
+  </si>
+  <si>
+    <t>Is Featured</t>
+  </si>
+  <si>
+    <t>BOLOGNA HB Executive Chair</t>
+  </si>
+  <si>
+    <t>SC0015</t>
+  </si>
+  <si>
+    <t>Office Chairs</t>
+  </si>
+  <si>
+    <t>Executive Chairs</t>
+  </si>
+  <si>
+    <t>Ergohuman</t>
+  </si>
+  <si>
+    <t>High-back leather executive chair. Unique curved backrest with lumbar support, height-adjustable backrest, synchro-tilt mechanism with seat slide, fixed chrome aluminium armrest with PU arm pad, aluminium base with PU castors.</t>
+  </si>
+  <si>
+    <t>Brown:4, Black:10</t>
+  </si>
+  <si>
+    <t>79x70x118cm</t>
+  </si>
+  <si>
+    <t>Genuine Leather</t>
+  </si>
+  <si>
+    <t>https://photos.app.goo.gl/K1bBRxTDsT98mAfe8, https://photos.app.goo.gl/71XCvy8U3r1WihTE7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13.5"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -132,10 +127,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
@@ -492,7 +485,7 @@
     <col min="12" max="12" width="44.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -500,78 +493,81 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2">
+        <v>5900</v>
+      </c>
+      <c r="H2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="18" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2">
-        <v>2400</v>
-      </c>
-      <c r="D2">
-        <v>15</v>
-      </c>
-      <c r="E2">
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" t="b">
         <v>1</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2" t="s">
-        <v>17</v>
-      </c>
-      <c r="L2" t="s">
-        <v>18</v>
+      <c r="M2" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:E1 A2:D2 G1:L1 H2:L2" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>